<commit_message>
This is an update that contains the refactored code and the original code in comments
</commit_message>
<xml_diff>
--- a/Excel Files/Boston_13x5x1.xlsx
+++ b/Excel Files/Boston_13x5x1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\colem\SummerResearch2021\Excel Files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E32151F1-C231-4E95-B04E-ADD00156530D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFBFF0C8-052C-453A-B6D2-1F20ABFACB0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -657,7 +657,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Boston_13x5x1!$A$5</c:f>
+              <c:f>Boston_13x5x1!$A$8</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -854,162 +854,162 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Boston_13x5x1!$B$5:$AZ$5</c:f>
+              <c:f>Boston_13x5x1!$B$8:$AZ$8</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="51"/>
                 <c:pt idx="0">
-                  <c:v>28.371730583823101</c:v>
+                  <c:v>57.974608418926699</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>18.3010542359523</c:v>
+                  <c:v>18.707524225002899</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>21.017375120394</c:v>
+                  <c:v>15.5308846339789</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>13.4764458180244</c:v>
+                  <c:v>14.5444310293418</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>14.8001917905372</c:v>
+                  <c:v>14.7644027944751</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>12.8763549239405</c:v>
+                  <c:v>16.886737367150399</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>13.252242591271299</c:v>
+                  <c:v>15.423952320765199</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>12.392325807200599</c:v>
+                  <c:v>14.779971880022</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>16.899065637843901</c:v>
+                  <c:v>16.3989502514337</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>12.404008165405701</c:v>
+                  <c:v>16.314455113259498</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>11.868995730586001</c:v>
+                  <c:v>14.1297896284951</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>12.824274243561501</c:v>
+                  <c:v>16.2439851601372</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>13.0066608588245</c:v>
+                  <c:v>13.502986142850901</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>13.189014686897799</c:v>
+                  <c:v>13.833243409928301</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>14.132201838055099</c:v>
+                  <c:v>14.541278147556101</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>12.735366089718701</c:v>
+                  <c:v>14.103209830183999</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>16.257431120952301</c:v>
+                  <c:v>15.2187117416573</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>11.037386862669999</c:v>
+                  <c:v>20.9502504270876</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>13.2975548120239</c:v>
+                  <c:v>14.464192157031199</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>12.033759084041399</c:v>
+                  <c:v>13.458323334170499</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>11.2654072761708</c:v>
+                  <c:v>12.949336899854799</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>11.393636816420701</c:v>
+                  <c:v>14.740237213249801</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>10.943307807352401</c:v>
+                  <c:v>13.4959259110136</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>14.3911703891938</c:v>
+                  <c:v>14.9028559594997</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>10.872149230287899</c:v>
+                  <c:v>13.460019471480701</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>12.137554112452101</c:v>
+                  <c:v>14.730353798074701</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>11.618345155064301</c:v>
+                  <c:v>13.8609202750006</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>11.3600743739007</c:v>
+                  <c:v>12.944896368130101</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>13.7589383494964</c:v>
+                  <c:v>14.156798753723001</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>11.0078464639502</c:v>
+                  <c:v>13.179887838253601</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>10.833294662817799</c:v>
+                  <c:v>13.3453810296421</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>12.2443197759127</c:v>
+                  <c:v>16.368013037093601</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>10.7697497902533</c:v>
+                  <c:v>13.760233321335701</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>11.299473636441901</c:v>
+                  <c:v>15.042563828553</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>11.1573697710836</c:v>
+                  <c:v>15.9097902356002</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>13.1356531285795</c:v>
+                  <c:v>12.6576172967634</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>11.506128632409901</c:v>
+                  <c:v>12.502618360161</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>10.498755561169901</c:v>
+                  <c:v>14.300019367615199</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>11.146527858720001</c:v>
+                  <c:v>12.4511270442725</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>11.0158794044963</c:v>
+                  <c:v>16.037542480075501</c:v>
                 </c:pt>
                 <c:pt idx="40">
-                  <c:v>14.333639217334699</c:v>
+                  <c:v>14.063282188287401</c:v>
                 </c:pt>
                 <c:pt idx="41">
-                  <c:v>11.2394051907931</c:v>
+                  <c:v>15.2564697506765</c:v>
                 </c:pt>
                 <c:pt idx="42">
-                  <c:v>11.5270318768293</c:v>
+                  <c:v>14.562402796039899</c:v>
                 </c:pt>
                 <c:pt idx="43">
-                  <c:v>10.892942927172699</c:v>
+                  <c:v>12.1863448989074</c:v>
                 </c:pt>
                 <c:pt idx="44">
-                  <c:v>13.324122754462</c:v>
+                  <c:v>14.163012102586301</c:v>
                 </c:pt>
                 <c:pt idx="45">
-                  <c:v>11.418114274008699</c:v>
+                  <c:v>12.344907957408701</c:v>
                 </c:pt>
                 <c:pt idx="46">
-                  <c:v>11.543957473133799</c:v>
+                  <c:v>14.1637762900439</c:v>
                 </c:pt>
                 <c:pt idx="47">
-                  <c:v>10.641823139936299</c:v>
+                  <c:v>13.5097314071278</c:v>
                 </c:pt>
                 <c:pt idx="48">
-                  <c:v>11.418729565644499</c:v>
+                  <c:v>12.625933266582299</c:v>
                 </c:pt>
                 <c:pt idx="49">
-                  <c:v>11.860330182109401</c:v>
+                  <c:v>12.6286106587978</c:v>
                 </c:pt>
                 <c:pt idx="50">
-                  <c:v>11.1230778242605</c:v>
+                  <c:v>11.5413837888718</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1026,7 +1026,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>Boston_13x5x1!$A$6</c:f>
+              <c:f>Boston_13x5x1!$A$9</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1223,162 +1223,162 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Boston_13x5x1!$B$6:$AZ$6</c:f>
+              <c:f>Boston_13x5x1!$B$9:$AZ$9</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="51"/>
                 <c:pt idx="0">
-                  <c:v>32.981437855146098</c:v>
+                  <c:v>47.636968167849297</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>21.667701002042001</c:v>
+                  <c:v>18.606016450936298</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>25.846749302462399</c:v>
+                  <c:v>14.7987479834387</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>17.484911446285601</c:v>
+                  <c:v>13.9840868307856</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>20.2742723662675</c:v>
+                  <c:v>15.1983126857765</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>14.716806140525501</c:v>
+                  <c:v>15.928254111656999</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>14.6196912355775</c:v>
+                  <c:v>15.2307969605822</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>15.0047485633698</c:v>
+                  <c:v>15.1402715762729</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>21.865861179917601</c:v>
+                  <c:v>14.136390500561999</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>14.4810580558156</c:v>
+                  <c:v>16.8896925135024</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>15.4503896442026</c:v>
+                  <c:v>13.162558599878899</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>17.134787232826898</c:v>
+                  <c:v>16.651379834126399</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>17.301193730334901</c:v>
+                  <c:v>13.384416573270901</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>16.688842909015101</c:v>
+                  <c:v>12.549686635193099</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>19.2150594022653</c:v>
+                  <c:v>14.156642836535999</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>16.880775523368399</c:v>
+                  <c:v>13.2739262549382</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>21.698368068557599</c:v>
+                  <c:v>13.9835490331825</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>13.525200595809601</c:v>
+                  <c:v>21.299965478587701</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>16.904742945703301</c:v>
+                  <c:v>14.3474352945903</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>15.18459693176</c:v>
+                  <c:v>13.514171224621199</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>14.2479749669815</c:v>
+                  <c:v>12.446697314799099</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>14.253064493058201</c:v>
+                  <c:v>14.5082292408597</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>13.7995255355416</c:v>
+                  <c:v>13.653232273541301</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>19.924855869420501</c:v>
+                  <c:v>15.803474639747099</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>13.497167891643</c:v>
+                  <c:v>13.0773082835187</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>15.7174820361501</c:v>
+                  <c:v>14.0167755092123</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>15.7271571518367</c:v>
+                  <c:v>13.5690931485825</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>14.863543412001601</c:v>
+                  <c:v>12.236390522307801</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>14.718265704628999</c:v>
+                  <c:v>14.417143853412901</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>14.560496884033</c:v>
+                  <c:v>12.4062999304805</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>13.821247298552599</c:v>
+                  <c:v>12.7049542589425</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>15.753107320721201</c:v>
+                  <c:v>16.987454607244398</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>14.1203635961717</c:v>
+                  <c:v>15.0094121544907</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>14.5814390860962</c:v>
+                  <c:v>16.301436399606001</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>13.479591005169</c:v>
+                  <c:v>17.013336099056598</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>17.483038547900701</c:v>
+                  <c:v>12.7210935341223</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>14.9240464746757</c:v>
+                  <c:v>12.86565567403</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>13.6149218312845</c:v>
+                  <c:v>14.6030529302085</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>15.456061279991699</c:v>
+                  <c:v>13.2607166038608</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>14.070767313463</c:v>
+                  <c:v>15.448996040898701</c:v>
                 </c:pt>
                 <c:pt idx="40">
-                  <c:v>19.6461627040492</c:v>
+                  <c:v>15.156445837474401</c:v>
                 </c:pt>
                 <c:pt idx="41">
-                  <c:v>15.253353683642301</c:v>
+                  <c:v>15.303212006393199</c:v>
                 </c:pt>
                 <c:pt idx="42">
-                  <c:v>14.850880429823899</c:v>
+                  <c:v>14.5831248752921</c:v>
                 </c:pt>
                 <c:pt idx="43">
-                  <c:v>13.395110130872601</c:v>
+                  <c:v>12.4062421598424</c:v>
                 </c:pt>
                 <c:pt idx="44">
-                  <c:v>17.328046807423199</c:v>
+                  <c:v>14.2912999537769</c:v>
                 </c:pt>
                 <c:pt idx="45">
-                  <c:v>15.7345783073843</c:v>
+                  <c:v>13.032808776182501</c:v>
                 </c:pt>
                 <c:pt idx="46">
-                  <c:v>15.733316512954399</c:v>
+                  <c:v>15.6710767326667</c:v>
                 </c:pt>
                 <c:pt idx="47">
-                  <c:v>14.022944432445801</c:v>
+                  <c:v>14.7853032859383</c:v>
                 </c:pt>
                 <c:pt idx="48">
-                  <c:v>15.144040025532499</c:v>
+                  <c:v>13.9731760699218</c:v>
                 </c:pt>
                 <c:pt idx="49">
-                  <c:v>16.250152484900202</c:v>
+                  <c:v>12.548081852360101</c:v>
                 </c:pt>
                 <c:pt idx="50">
-                  <c:v>15.770365043863199</c:v>
+                  <c:v>11.8763121291293</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1395,7 +1395,7 @@
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>Boston_13x5x1!$A$7</c:f>
+              <c:f>Boston_13x5x1!$A$10</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1592,162 +1592,162 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Boston_13x5x1!$B$7:$AZ$7</c:f>
+              <c:f>Boston_13x5x1!$B$10:$AZ$10</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="51"/>
                 <c:pt idx="0">
-                  <c:v>25.749623323088699</c:v>
+                  <c:v>43.917774220053701</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>17.471006750560999</c:v>
+                  <c:v>19.01695404809</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>23.3577308708395</c:v>
+                  <c:v>16.340465154323098</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>16.064003642805801</c:v>
+                  <c:v>16.026560076507501</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>15.9420289494568</c:v>
+                  <c:v>16.010098581785801</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>14.495475516641401</c:v>
+                  <c:v>16.881394729802601</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>14.716556362970399</c:v>
+                  <c:v>16.5872795051759</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>14.0832243110127</c:v>
+                  <c:v>15.645353746148</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>21.067845824819301</c:v>
+                  <c:v>15.396212045736799</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>14.562188190181701</c:v>
+                  <c:v>17.653766586260002</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>14.806282732595699</c:v>
+                  <c:v>14.1371421284682</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>14.730121259033099</c:v>
+                  <c:v>16.865305602139401</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>15.0371389414356</c:v>
+                  <c:v>14.519622691355099</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>15.6092749629961</c:v>
+                  <c:v>14.172179348501</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>17.180118978727901</c:v>
+                  <c:v>14.216344896519701</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>15.4108168013368</c:v>
+                  <c:v>14.673591725214401</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>21.541179780834501</c:v>
+                  <c:v>14.2378004624201</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>12.824616300484101</c:v>
+                  <c:v>20.972526345996101</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>15.781802566499501</c:v>
+                  <c:v>15.352759142545301</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>13.806057574168101</c:v>
+                  <c:v>13.8678568797036</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>13.2580217259185</c:v>
+                  <c:v>13.306051183326799</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>13.6399611185601</c:v>
+                  <c:v>14.4178977756319</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>13.2398729120696</c:v>
+                  <c:v>14.4673479433027</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>17.502672244134001</c:v>
+                  <c:v>16.840976338669201</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>13.0177786626372</c:v>
+                  <c:v>13.712663194982699</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>14.879043078069801</c:v>
+                  <c:v>13.5435282389492</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>13.490231179554</c:v>
+                  <c:v>13.9901159335536</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>13.542879452203</c:v>
+                  <c:v>12.9793431812944</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>14.524955200378001</c:v>
+                  <c:v>15.576760240918</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>13.071020930463201</c:v>
+                  <c:v>12.847984010158999</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>13.476840750419299</c:v>
+                  <c:v>12.873316126498199</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>14.215339739177599</c:v>
+                  <c:v>16.813361623836599</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>13.1784573555816</c:v>
+                  <c:v>15.515645148575899</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>13.7707396966657</c:v>
+                  <c:v>17.086991880205201</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>13.7519090782239</c:v>
+                  <c:v>17.8329259998239</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>15.060888115134</c:v>
+                  <c:v>12.5364633491875</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>13.7857029973688</c:v>
+                  <c:v>13.419505376517399</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>12.804295612298899</c:v>
+                  <c:v>14.668614924906899</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>13.559654102212701</c:v>
+                  <c:v>13.5058462801648</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>13.4678412449967</c:v>
+                  <c:v>14.6737225007881</c:v>
                 </c:pt>
                 <c:pt idx="40">
-                  <c:v>18.628596204344699</c:v>
+                  <c:v>16.6214023300722</c:v>
                 </c:pt>
                 <c:pt idx="41">
-                  <c:v>13.8385587511252</c:v>
+                  <c:v>13.325929644391699</c:v>
                 </c:pt>
                 <c:pt idx="42">
-                  <c:v>13.6668376489457</c:v>
+                  <c:v>13.354781682568699</c:v>
                 </c:pt>
                 <c:pt idx="43">
-                  <c:v>13.421671468273701</c:v>
+                  <c:v>12.084154577272001</c:v>
                 </c:pt>
                 <c:pt idx="44">
-                  <c:v>14.647371281669599</c:v>
+                  <c:v>12.3809720602132</c:v>
                 </c:pt>
                 <c:pt idx="45">
-                  <c:v>14.3769916236608</c:v>
+                  <c:v>13.678114862077299</c:v>
                 </c:pt>
                 <c:pt idx="46">
-                  <c:v>14.8026337588334</c:v>
+                  <c:v>14.5960194570513</c:v>
                 </c:pt>
                 <c:pt idx="47">
-                  <c:v>13.054395684981699</c:v>
+                  <c:v>13.9927135514853</c:v>
                 </c:pt>
                 <c:pt idx="48">
-                  <c:v>14.092333163824501</c:v>
+                  <c:v>14.5856511002372</c:v>
                 </c:pt>
                 <c:pt idx="49">
-                  <c:v>14.117886478429901</c:v>
+                  <c:v>12.0568841633168</c:v>
                 </c:pt>
                 <c:pt idx="50">
-                  <c:v>14.0012840248886</c:v>
+                  <c:v>12.0059275206289</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2653,15 +2653,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>32</xdr:col>
-      <xdr:colOff>264794</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>40005</xdr:rowOff>
+      <xdr:colOff>470534</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>50</xdr:col>
-      <xdr:colOff>40004</xdr:colOff>
-      <xdr:row>34</xdr:row>
-      <xdr:rowOff>173355</xdr:rowOff>
+      <xdr:colOff>245744</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>180975</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>

</xml_diff>